<commit_message>
Fix invalid Excel formula ranges in generated workbook
</commit_message>
<xml_diff>
--- a/prevent_calculator.xlsx
+++ b/prevent_calculator.xlsx
@@ -1061,23 +1061,23 @@
         <v>13</v>
       </c>
       <c r="E6" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$B$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$C$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$B$2:$B$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$C$2:$C$33")))))</f>
         <v>0.14683939095644824</v>
       </c>
       <c r="F6" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$L$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$M$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$L$2:$L$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$M$2:$M$33")))))</f>
         <v>0.15992298123481016</v>
       </c>
       <c r="G6" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$V$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$W$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$V$2:$V$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$W$2:$W$33")))))</f>
         <v>0.13586705019403117</v>
       </c>
       <c r="H6" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AF$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AG$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AF$2:$AF$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AG$2:$AG$33")))))</f>
         <v>0.1565456427896422</v>
       </c>
       <c r="I6" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AP$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AQ$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AP$2:$AP$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AQ$2:$AQ$33")))))</f>
         <v>0.15597624665790258</v>
       </c>
     </row>
@@ -1092,23 +1092,23 @@
         <v>15</v>
       </c>
       <c r="E7" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$D$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$E$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$D$2:$D$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$E$2:$E$33")))))</f>
         <v>0.09195089753632874</v>
       </c>
       <c r="F7" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$N$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$O$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$N$2:$N$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$O$2:$O$33")))))</f>
         <v>0.09944272308807872</v>
       </c>
       <c r="G7" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$X$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$Y$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$X$2:$X$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$Y$2:$Y$33")))))</f>
         <v>0.08349803993883279</v>
       </c>
       <c r="H7" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AH$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AI$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AH$2:$AH$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AI$2:$AI$33")))))</f>
         <v>0.10034803473666952</v>
       </c>
       <c r="I7" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AR$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AS$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AR$2:$AR$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AS$2:$AS$33")))))</f>
         <v>0.09638939920734978</v>
       </c>
     </row>
@@ -1123,23 +1123,23 @@
         <v>17</v>
       </c>
       <c r="E8" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$F$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$G$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$F$2:$F$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$G$2:$G$33")))))</f>
         <v>0.08056096777914257</v>
       </c>
       <c r="F8" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$P$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$Q$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$P$2:$P$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$Q$2:$Q$33")))))</f>
         <v>0.0893240911620721</v>
       </c>
       <c r="G8" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$Z$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AA$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$Z$2:$Z$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AA$2:$AA$33")))))</f>
         <v>0.08056689661287753</v>
       </c>
       <c r="H8" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AJ$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AK$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AJ$2:$AJ$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AK$2:$AK$33")))))</f>
         <v>0.08862750903165648</v>
       </c>
       <c r="I8" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AT$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AU$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AT$2:$AT$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AU$2:$AU$33")))))</f>
         <v>0.09265294260535863</v>
       </c>
     </row>
@@ -1154,23 +1154,23 @@
         <v>19</v>
       </c>
       <c r="E9" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$H$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$I$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$H$2:$H$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$I$2:$I$33")))))</f>
         <v>0.04409666763894401</v>
       </c>
       <c r="F9" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$R$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$S$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$R$2:$R$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$S$2:$S$33")))))</f>
         <v>0.04808574158607073</v>
       </c>
       <c r="G9" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AB$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AC$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AB$2:$AB$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AC$2:$AC$33")))))</f>
         <v>0.04108306816495741</v>
       </c>
       <c r="H9" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AL$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AM$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AL$2:$AL$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AM$2:$AM$33")))))</f>
         <v>0.04815889193744638</v>
       </c>
       <c r="I9" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AV$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AW$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AV$2:$AV$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AW$2:$AW$33")))))</f>
         <v>0.04736405897141795</v>
       </c>
     </row>
@@ -1185,23 +1185,23 @@
         <v>22</v>
       </c>
       <c r="E10" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$J$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$K$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$J$2:$J$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$K$2:$K$33")))))</f>
         <v>0.054007794606351675</v>
       </c>
       <c r="F10" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$T$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$U$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$T$2:$T$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$U$2:$U$33")))))</f>
         <v>0.058572838843231674</v>
       </c>
       <c r="G10" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AD$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AE$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AD$2:$AD$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AE$2:$AE$33")))))</f>
         <v>0.04570245682380386</v>
       </c>
       <c r="H10" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AN$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AO$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AN$2:$AN$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AO$2:$AO$33")))))</f>
         <v>0.05843632432037109</v>
       </c>
       <c r="I10" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AX$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AY$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AX$2:$AX$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AY$2:$AY$33")))))</f>
         <v>0.05369190874491909</v>
       </c>
     </row>
@@ -1269,23 +1269,23 @@
         <v>13</v>
       </c>
       <c r="E15" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$AZ$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BA$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$AZ$2:$AZ$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BA$2:$BA$33")))))</f>
         <v>0.5298503870635785</v>
       </c>
       <c r="F15" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BJ$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BK$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BJ$2:$BJ$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BK$2:$BK$33")))))</f>
         <v>0.5415637333921166</v>
       </c>
       <c r="G15" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BT$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BU$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BT$2:$BT$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BU$2:$BU$33")))))</f>
         <v>0.5006211918945594</v>
       </c>
       <c r="H15" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CD$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CE$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CD$2:$CD$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CE$2:$CE$33")))))</f>
         <v>0.534703048887485</v>
       </c>
       <c r="I15" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CN$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CO$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CN$2:$CN$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CO$2:$CO$33")))))</f>
         <v>0.5196551757355707</v>
       </c>
     </row>
@@ -1300,23 +1300,23 @@
         <v>15</v>
       </c>
       <c r="E16" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BB$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BC$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BB$2:$BB$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BC$2:$BC$33")))))</f>
         <v>0.3542551988690411</v>
       </c>
       <c r="F16" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BL$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BM$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BL$2:$BL$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BM$2:$BM$33")))))</f>
         <v>0.36322352848120315</v>
       </c>
       <c r="G16" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BV$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BW$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BV$2:$BV$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BW$2:$BW$33")))))</f>
         <v>0.32238789906475523</v>
       </c>
       <c r="H16" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CF$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CG$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CF$2:$CF$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CG$2:$CG$33")))))</f>
         <v>0.36695490488059235</v>
       </c>
       <c r="I16" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CP$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CQ$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CP$2:$CP$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CQ$2:$CQ$33")))))</f>
         <v>0.3437137287596968</v>
       </c>
     </row>
@@ -1331,23 +1331,23 @@
         <v>17</v>
       </c>
       <c r="E17" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BD$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BE$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BD$2:$BD$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BE$2:$BE$33")))))</f>
         <v>0.38960226711066315</v>
       </c>
       <c r="F17" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BN$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BO$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BN$2:$BN$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BO$2:$BO$33")))))</f>
         <v>0.4065973332722868</v>
       </c>
       <c r="G17" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BX$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BY$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BX$2:$BX$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BY$2:$BY$33")))))</f>
         <v>0.38921345951338443</v>
       </c>
       <c r="H17" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CH$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CI$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CH$2:$CH$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CI$2:$CI$33")))))</f>
         <v>0.40434948980611823</v>
       </c>
       <c r="I17" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CR$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CS$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CR$2:$CR$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CS$2:$CS$33")))))</f>
         <v>0.40502302842081933</v>
       </c>
     </row>
@@ -1362,23 +1362,23 @@
         <v>19</v>
       </c>
       <c r="E18" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BF$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BG$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BF$2:$BF$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BG$2:$BG$33")))))</f>
         <v>0.19818169195864557</v>
       </c>
       <c r="F18" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BP$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BQ$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BP$2:$BP$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BQ$2:$BQ$33")))))</f>
         <v>0.20590405573947437</v>
       </c>
       <c r="G18" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BZ$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CA$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BZ$2:$BZ$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CA$2:$CA$33")))))</f>
         <v>0.18211219465582462</v>
       </c>
       <c r="H18" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CJ$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CK$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CJ$2:$CJ$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CK$2:$CK$33")))))</f>
         <v>0.21055631637332342</v>
       </c>
       <c r="I18" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CT$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CU$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CT$2:$CT$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CU$2:$CU$33")))))</f>
         <v>0.1981291300451217</v>
       </c>
     </row>
@@ -1387,23 +1387,23 @@
         <v>22</v>
       </c>
       <c r="E19" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BH$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BI$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BH$2:$BH$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BI$2:$BI$33")))))</f>
         <v>0.22100434259063864</v>
       </c>
       <c r="F19" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BR$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$BS$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BR$2:$BR$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$BS$2:$BS$33")))))</f>
         <v>0.2288049834564067</v>
       </c>
       <c r="G19" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CB$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CC$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CB$2:$CB$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CC$2:$CC$33")))))</f>
         <v>0.18828025719410832</v>
       </c>
       <c r="H19" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CL$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CM$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CL$2:$CL$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CM$2:$CM$33")))))</f>
         <v>0.23181015716946407</v>
       </c>
       <c r="I19" s="6">
-        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CV$2:$33))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,Coefficients!$CW$2:$33))))</f>
+        <f>IF($B$5="Women",1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CV$2:$CV$33")))),1/(1+EXP(-SUMPRODUCT(Engine!$B$2:$B$33,INDIRECT("Coefficients!$CW$2:$CW$33")))))</f>
         <v>0.20767427433359964</v>
       </c>
     </row>

</xml_diff>